<commit_message>
Audit et nettoyage terminé
</commit_message>
<xml_diff>
--- a/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
+++ b/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Documents/Formation AI Engineer OC/Projet_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA4C521C-213B-A743-9D7F-48EA1F65A2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0068F7B-D0DA-AD49-A771-D782B6E289E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="167">
   <si>
     <t>#</t>
   </si>
@@ -359,12 +359,6 @@
   </si>
   <si>
     <t>Audit du dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimensions </t>
-  </si>
-  <si>
-    <t>3376, 46</t>
   </si>
   <si>
     <t>Lignes en doublon</t>
@@ -416,9 +410,6 @@
     <t>FE1</t>
   </si>
   <si>
-    <t xml:space="preserve">is_multi_type </t>
-  </si>
-  <si>
     <t>Booléen 0/1</t>
   </si>
   <si>
@@ -450,9 +441,6 @@
   </si>
   <si>
     <t xml:space="preserve">L'identifiant unique n'est pas pertinent a garder car nous ne souhiatons pas identifier un batiment en particulier </t>
-  </si>
-  <si>
-    <t>nb de lignes sans habitation</t>
   </si>
   <si>
     <t>Pas utile a garder pour l'analyse mais nécessaire pour filtrer les habitations pour ne pas les traiter</t>
@@ -579,12 +567,55 @@
   <si>
     <t>Définit l'age du batiment (2026-YearBuilt)</t>
   </si>
+  <si>
+    <t xml:space="preserve">Lignes / Colonnes </t>
+  </si>
+  <si>
+    <t>3376 /  46</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pas exploitables car presque toutes vides 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF333333"/>
+        <rFont val="Segoe UI"/>
+      </rPr>
+      <t>building_consumption['Outlier'].value_counts(dropna= False)</t>
+    </r>
+  </si>
+  <si>
+    <t>Lignes sans résidentiel</t>
+  </si>
+  <si>
+    <t>Uniquement les colonnes nécessaires pour ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nouvelles dimentions 
+Lignes / Colonnes </t>
+  </si>
+  <si>
+    <t>1668 / 15</t>
+  </si>
+  <si>
+    <t>Pour calculer FE2</t>
+  </si>
+  <si>
+    <t>Calculée a partir du nb de valeurs dans la variable "YearBuilt"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is_multi_type </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -637,6 +668,12 @@
     <font>
       <b/>
       <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color rgb="FF333333"/>
       <name val="Segoe UI"/>
     </font>
@@ -758,7 +795,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -796,44 +833,49 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1138,7 +1180,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N58"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -1158,10 +1201,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="35" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="14"/>
+      <c r="B1" s="24"/>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,31 +1218,31 @@
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>122</v>
+      <c r="I1" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>120</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="M1" s="26" t="s">
-        <v>135</v>
+        <v>137</v>
+      </c>
+      <c r="M1" s="22" t="s">
+        <v>132</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>112</v>
+        <v>157</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>113</v>
+        <v>158</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -1211,23 +1254,23 @@
         <v>5</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L2" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-    </row>
-    <row r="3" spans="1:14" ht="59" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L2" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+    </row>
+    <row r="3" spans="1:14" ht="59" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B3" s="8">
         <v>0</v>
@@ -1242,23 +1285,28 @@
         <v>8</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-    </row>
-    <row r="4" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>142</v>
+      <c r="I3" s="15"/>
+      <c r="J3" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L3" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+    </row>
+    <row r="4" spans="1:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4" s="8">
+        <v>1668</v>
       </c>
       <c r="D4" s="3">
         <v>3</v>
@@ -1270,21 +1318,27 @@
         <v>11</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L4" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-    </row>
-    <row r="5" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+    </row>
+    <row r="5" spans="1:14" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="8">
+        <v>15</v>
+      </c>
       <c r="D5" s="5">
         <v>4</v>
       </c>
@@ -1295,21 +1349,27 @@
         <v>14</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L5" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-    </row>
-    <row r="6" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L5" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+    </row>
+    <row r="6" spans="1:14" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B6" t="s">
+        <v>163</v>
+      </c>
       <c r="D6" s="3">
         <v>5</v>
       </c>
@@ -1320,21 +1380,21 @@
         <v>16</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L6" s="20" t="s">
-        <v>145</v>
-      </c>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-    </row>
-    <row r="7" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L6" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+    </row>
+    <row r="7" spans="1:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D7" s="5">
         <v>6</v>
       </c>
@@ -1345,21 +1405,21 @@
         <v>18</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L7" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-    </row>
-    <row r="8" spans="1:14" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+    </row>
+    <row r="8" spans="1:14" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D8" s="3">
         <v>7</v>
       </c>
@@ -1370,21 +1430,21 @@
         <v>20</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L8" s="20" t="s">
-        <v>148</v>
-      </c>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-    </row>
-    <row r="9" spans="1:14" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
+    </row>
+    <row r="9" spans="1:14" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D9" s="5">
         <v>8</v>
       </c>
@@ -1395,21 +1455,21 @@
         <v>22</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L9" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-    </row>
-    <row r="10" spans="1:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L9" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+    </row>
+    <row r="10" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D10" s="3">
         <v>9</v>
       </c>
@@ -1420,21 +1480,21 @@
         <v>24</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L10" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
-    </row>
-    <row r="11" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L10" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+    </row>
+    <row r="11" spans="1:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D11" s="5">
         <v>10</v>
       </c>
@@ -1445,21 +1505,21 @@
         <v>26</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L11" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-    </row>
-    <row r="12" spans="1:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L11" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+    </row>
+    <row r="12" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D12" s="3">
         <v>11</v>
       </c>
@@ -1470,21 +1530,21 @@
         <v>28</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L12" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="M12" s="20"/>
-      <c r="N12" s="20"/>
-    </row>
-    <row r="13" spans="1:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+    </row>
+    <row r="13" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D13" s="5">
         <v>12</v>
       </c>
@@ -1495,21 +1555,21 @@
         <v>31</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="M13" s="20"/>
-      <c r="N13" s="20"/>
-    </row>
-    <row r="14" spans="1:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
+    </row>
+    <row r="14" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D14" s="3">
         <v>13</v>
       </c>
@@ -1520,21 +1580,21 @@
         <v>33</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L14" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="M14" s="20"/>
-      <c r="N14" s="20"/>
-    </row>
-    <row r="15" spans="1:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L14" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
+    </row>
+    <row r="15" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D15" s="5">
         <v>14</v>
       </c>
@@ -1545,19 +1605,19 @@
         <v>36</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L15" s="20" t="s">
-        <v>151</v>
-      </c>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L15" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
     </row>
     <row r="16" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="3">
@@ -1570,20 +1630,20 @@
         <v>38</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="18" t="s">
+      <c r="H16" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="I16" s="19"/>
-      <c r="J16" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="K16" s="20" t="s">
+      <c r="I16" s="17"/>
+      <c r="J16" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L16" s="18"/>
+      <c r="M16" s="18"/>
+      <c r="N16" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="17" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1597,20 +1657,20 @@
         <v>40</v>
       </c>
       <c r="G17" s="2"/>
-      <c r="H17" s="18" t="s">
+      <c r="H17" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="I17" s="19"/>
-      <c r="J17" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="K17" s="20" t="s">
+      <c r="I17" s="17"/>
+      <c r="J17" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L17" s="20"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="18" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1624,20 +1684,20 @@
         <v>42</v>
       </c>
       <c r="G18" s="2"/>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="19"/>
-      <c r="J18" s="20" t="s">
-        <v>126</v>
-      </c>
-      <c r="K18" s="20" t="s">
+      <c r="I18" s="17"/>
+      <c r="J18" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="19" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
@@ -1651,18 +1711,18 @@
         <v>44</v>
       </c>
       <c r="G19" s="2"/>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="I19" s="19"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20" t="s">
+      <c r="I19" s="17"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L19" s="18"/>
+      <c r="M19" s="18"/>
+      <c r="N19" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="20" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1676,18 +1736,18 @@
         <v>47</v>
       </c>
       <c r="G20" s="2"/>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="20"/>
-      <c r="K20" s="20" t="s">
+      <c r="I20" s="17"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L20" s="20"/>
-      <c r="M20" s="20"/>
-      <c r="N20" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="21" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1701,18 +1761,18 @@
         <v>49</v>
       </c>
       <c r="G21" s="2"/>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="I21" s="19"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20" t="s">
+      <c r="I21" s="17"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L21" s="18"/>
+      <c r="M21" s="18"/>
+      <c r="N21" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="22" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1726,27 +1786,25 @@
         <v>51</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="J22" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="K22" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="L22" s="20"/>
-      <c r="M22" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="N22" s="20" t="s">
+      <c r="H22" s="16" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="23" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I22" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L22" s="18"/>
+      <c r="M22" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="N22" s="18"/>
+    </row>
+    <row r="23" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D23" s="5">
         <v>22</v>
       </c>
@@ -1757,21 +1815,21 @@
         <v>53</v>
       </c>
       <c r="G23" s="2"/>
-      <c r="H23" s="16" t="s">
+      <c r="H23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L23" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M23" s="20"/>
-      <c r="N23" s="20"/>
-    </row>
-    <row r="24" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L23" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M23" s="18"/>
+      <c r="N23" s="18"/>
+    </row>
+    <row r="24" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D24" s="3">
         <v>23</v>
       </c>
@@ -1782,21 +1840,21 @@
         <v>55</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="16" t="s">
+      <c r="H24" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L24" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M24" s="20"/>
-      <c r="N24" s="20"/>
-    </row>
-    <row r="25" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L24" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M24" s="18"/>
+      <c r="N24" s="18"/>
+    </row>
+    <row r="25" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D25" s="5">
         <v>24</v>
       </c>
@@ -1807,21 +1865,21 @@
         <v>57</v>
       </c>
       <c r="G25" s="2"/>
-      <c r="H25" s="16" t="s">
+      <c r="H25" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="17"/>
-      <c r="J25" s="17"/>
-      <c r="K25" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L25" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M25" s="20"/>
-      <c r="N25" s="20"/>
-    </row>
-    <row r="26" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L25" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
+    </row>
+    <row r="26" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D26" s="3">
         <v>25</v>
       </c>
@@ -1832,21 +1890,21 @@
         <v>59</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="16" t="s">
+      <c r="H26" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="I26" s="17"/>
-      <c r="J26" s="17"/>
-      <c r="K26" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L26" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M26" s="20"/>
-      <c r="N26" s="20"/>
-    </row>
-    <row r="27" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M26" s="18"/>
+      <c r="N26" s="18"/>
+    </row>
+    <row r="27" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D27" s="5">
         <v>26</v>
       </c>
@@ -1857,21 +1915,21 @@
         <v>61</v>
       </c>
       <c r="G27" s="2"/>
-      <c r="H27" s="16" t="s">
+      <c r="H27" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
-      <c r="K27" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L27" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M27" s="20"/>
-      <c r="N27" s="20"/>
-    </row>
-    <row r="28" spans="4:14" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+      <c r="K27" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L27" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
+    </row>
+    <row r="28" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D28" s="3">
         <v>27</v>
       </c>
@@ -1882,21 +1940,21 @@
         <v>63</v>
       </c>
       <c r="G28" s="2"/>
-      <c r="H28" s="16" t="s">
+      <c r="H28" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="I28" s="17"/>
-      <c r="J28" s="17"/>
-      <c r="K28" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L28" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-    </row>
-    <row r="29" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+      <c r="K28" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L28" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="M28" s="18"/>
+      <c r="N28" s="18"/>
+    </row>
+    <row r="29" spans="4:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D29" s="5">
         <v>28</v>
       </c>
@@ -1907,21 +1965,21 @@
         <v>65</v>
       </c>
       <c r="G29" s="2"/>
-      <c r="H29" s="16" t="s">
+      <c r="H29" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L29" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="M29" s="20"/>
-      <c r="N29" s="20"/>
-    </row>
-    <row r="30" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L29" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="M29" s="18"/>
+      <c r="N29" s="18"/>
+    </row>
+    <row r="30" spans="4:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D30" s="3">
         <v>29</v>
       </c>
@@ -1932,19 +1990,19 @@
         <v>68</v>
       </c>
       <c r="G30" s="2"/>
-      <c r="H30" s="16" t="s">
+      <c r="H30" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L30" s="20" t="s">
-        <v>150</v>
-      </c>
-      <c r="M30" s="20"/>
-      <c r="N30" s="20"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+      <c r="K30" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L30" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="M30" s="18"/>
+      <c r="N30" s="18"/>
     </row>
     <row r="31" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D31" s="5">
@@ -1957,21 +2015,21 @@
         <v>71</v>
       </c>
       <c r="G31" s="2"/>
-      <c r="H31" s="18" t="s">
+      <c r="H31" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="I31" s="19"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20" t="s">
+      <c r="I31" s="17"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L31" s="18"/>
+      <c r="M31" s="18"/>
+      <c r="N31" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L31" s="20"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="32" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D32" s="3">
         <v>31</v>
       </c>
@@ -1982,21 +2040,21 @@
         <v>74</v>
       </c>
       <c r="G32" s="2"/>
-      <c r="H32" s="16" t="s">
+      <c r="H32" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L32" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="M32" s="20"/>
-      <c r="N32" s="20"/>
-    </row>
-    <row r="33" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L32" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+    </row>
+    <row r="33" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D33" s="5">
         <v>32</v>
       </c>
@@ -2007,21 +2065,21 @@
         <v>76</v>
       </c>
       <c r="G33" s="2"/>
-      <c r="H33" s="16" t="s">
+      <c r="H33" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L33" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="M33" s="20"/>
-      <c r="N33" s="20"/>
-    </row>
-    <row r="34" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L33" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M33" s="18"/>
+      <c r="N33" s="18"/>
+    </row>
+    <row r="34" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D34" s="3">
         <v>33</v>
       </c>
@@ -2032,19 +2090,19 @@
         <v>78</v>
       </c>
       <c r="G34" s="2"/>
-      <c r="H34" s="16" t="s">
+      <c r="H34" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="I34" s="17"/>
-      <c r="J34" s="17"/>
-      <c r="K34" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L34" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="M34" s="20"/>
-      <c r="N34" s="20"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L34" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M34" s="18"/>
+      <c r="N34" s="18"/>
     </row>
     <row r="35" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D35" s="5">
@@ -2057,23 +2115,25 @@
         <v>80</v>
       </c>
       <c r="G35" s="2"/>
-      <c r="H35" s="18" t="s">
+      <c r="H35" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I35" s="19"/>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="L35" s="20"/>
-      <c r="M35" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="N35" s="20" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="36" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I35" s="17"/>
+      <c r="J35" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K35" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L35" s="18"/>
+      <c r="M35" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="N35" s="27" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="36" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D36" s="3">
         <v>35</v>
       </c>
@@ -2084,19 +2144,19 @@
         <v>83</v>
       </c>
       <c r="G36" s="2"/>
-      <c r="H36" s="16" t="s">
+      <c r="H36" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="I36" s="17"/>
-      <c r="J36" s="17"/>
-      <c r="K36" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L36" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="M36" s="20"/>
-      <c r="N36" s="20"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L36" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
     </row>
     <row r="37" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D37" s="5">
@@ -2109,21 +2169,23 @@
         <v>85</v>
       </c>
       <c r="G37" s="2"/>
-      <c r="H37" s="18" t="s">
+      <c r="H37" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I37" s="19"/>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20" t="s">
+      <c r="I37" s="17"/>
+      <c r="J37" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K37" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L37" s="18"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L37" s="20"/>
-      <c r="M37" s="20"/>
-      <c r="N37" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="38" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D38" s="3">
         <v>37</v>
       </c>
@@ -2134,19 +2196,19 @@
         <v>87</v>
       </c>
       <c r="G38" s="2"/>
-      <c r="H38" s="16" t="s">
+      <c r="H38" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L38" s="20" t="s">
-        <v>156</v>
-      </c>
-      <c r="M38" s="20"/>
-      <c r="N38" s="20"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L38" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
     </row>
     <row r="39" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D39" s="5">
@@ -2159,21 +2221,23 @@
         <v>90</v>
       </c>
       <c r="G39" s="2"/>
-      <c r="H39" s="18" t="s">
+      <c r="H39" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I39" s="19"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20" t="s">
+      <c r="I39" s="17"/>
+      <c r="J39" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K39" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="40" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D40" s="3">
         <v>39</v>
       </c>
@@ -2184,19 +2248,19 @@
         <v>92</v>
       </c>
       <c r="G40" s="2"/>
-      <c r="H40" s="16" t="s">
+      <c r="H40" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L40" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L40" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="M40" s="18"/>
+      <c r="N40" s="18"/>
     </row>
     <row r="41" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D41" s="5">
@@ -2209,18 +2273,20 @@
         <v>95</v>
       </c>
       <c r="G41" s="2"/>
-      <c r="H41" s="18" t="s">
+      <c r="H41" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I41" s="19"/>
-      <c r="J41" s="20"/>
-      <c r="K41" s="20" t="s">
+      <c r="I41" s="17"/>
+      <c r="J41" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="K41" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L41" s="20"/>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="42" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
@@ -2234,23 +2300,23 @@
         <v>97</v>
       </c>
       <c r="G42" s="2"/>
-      <c r="H42" s="18" t="s">
+      <c r="H42" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="I42" s="19"/>
-      <c r="J42" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="K42" s="20" t="s">
+      <c r="I42" s="17"/>
+      <c r="J42" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="K42" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L42" s="18"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="43" spans="4:14" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="4:14" ht="28" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D43" s="5">
         <v>42</v>
       </c>
@@ -2261,19 +2327,19 @@
         <v>100</v>
       </c>
       <c r="G43" s="2"/>
-      <c r="H43" s="16" t="s">
+      <c r="H43" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L43" s="20" t="s">
-        <v>158</v>
-      </c>
-      <c r="M43" s="20"/>
-      <c r="N43" s="20"/>
+      <c r="I43" s="15"/>
+      <c r="J43" s="15"/>
+      <c r="K43" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L43" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="M43" s="18"/>
+      <c r="N43" s="18"/>
     </row>
     <row r="44" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D44" s="3">
@@ -2286,25 +2352,25 @@
         <v>102</v>
       </c>
       <c r="G44" s="2"/>
-      <c r="H44" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="I44" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="J44" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="K44" s="20" t="s">
+      <c r="H44" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="J44" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="K44" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L44" s="18"/>
+      <c r="M44" s="18"/>
+      <c r="N44" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L44" s="20"/>
-      <c r="M44" s="20"/>
-      <c r="N44" s="20" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="45" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D45" s="5">
         <v>44</v>
       </c>
@@ -2315,20 +2381,22 @@
         <v>104</v>
       </c>
       <c r="G45" s="2"/>
-      <c r="H45" s="18" t="s">
+      <c r="H45" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="I45" s="19"/>
-      <c r="J45" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="K45" s="20" t="s">
+      <c r="I45" s="17"/>
+      <c r="J45" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="K45" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L45" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="M45" s="18"/>
+      <c r="N45" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="L45" s="20"/>
-      <c r="M45" s="20"/>
-      <c r="N45" s="20" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="46" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
@@ -2342,23 +2410,23 @@
         <v>106</v>
       </c>
       <c r="G46" s="2"/>
-      <c r="H46" s="18" t="s">
+      <c r="H46" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="I46" s="19"/>
-      <c r="J46" s="20"/>
-      <c r="K46" s="20" t="s">
+      <c r="I46" s="17"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L46" s="18"/>
+      <c r="M46" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="N46" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="L46" s="20"/>
-      <c r="M46" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="N46" s="20" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="47" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D47" s="5">
         <v>46</v>
       </c>
@@ -2369,19 +2437,19 @@
         <v>109</v>
       </c>
       <c r="G47" s="2"/>
-      <c r="H47" s="16" t="s">
+      <c r="H47" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17"/>
-      <c r="K47" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="L47" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="M47" s="20"/>
-      <c r="N47" s="20"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+      <c r="K47" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="L47" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
     </row>
     <row r="48" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
@@ -2397,140 +2465,86 @@
       <c r="N48" s="2"/>
     </row>
     <row r="49" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="23" t="s">
+      <c r="D49" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="E49" s="20" t="s">
+        <v>166</v>
+      </c>
+      <c r="F49" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="G49" s="2"/>
+      <c r="H49" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="J49" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="N49" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="E49" s="24" t="s">
-        <v>130</v>
-      </c>
-      <c r="F49" s="25" t="s">
-        <v>133</v>
-      </c>
-      <c r="G49" s="2"/>
-      <c r="H49" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="I49" s="21"/>
-      <c r="J49" s="20" t="s">
+    </row>
+    <row r="50" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D50" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="K49" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="L49" s="20"/>
-      <c r="M49" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="N49" s="20" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="50" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D50" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="E50" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="F50" s="25" t="s">
-        <v>160</v>
+      <c r="E50" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="F50" s="21" t="s">
+        <v>156</v>
       </c>
       <c r="G50" s="2"/>
-      <c r="H50" s="18" t="s">
+      <c r="H50" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="I50" s="21"/>
-      <c r="J50" s="22"/>
-      <c r="K50" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="L50" s="20"/>
-      <c r="M50" s="20" t="s">
-        <v>117</v>
-      </c>
-      <c r="N50" s="20" t="s">
-        <v>132</v>
+      <c r="J50" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="K50" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="N50" s="18" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="51" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G51" s="2"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="22"/>
-      <c r="K51" s="21"/>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
-      <c r="N51" s="21"/>
+      <c r="H51" s="25"/>
+      <c r="K51" s="26"/>
     </row>
     <row r="52" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G52" s="2"/>
-      <c r="H52" s="21"/>
-      <c r="I52" s="21"/>
-      <c r="J52" s="22"/>
-      <c r="K52" s="21"/>
-      <c r="L52" s="21"/>
-      <c r="M52" s="21"/>
-      <c r="N52" s="21"/>
     </row>
     <row r="53" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G53" s="2"/>
-      <c r="H53" s="21"/>
-      <c r="I53" s="21"/>
-      <c r="J53" s="22"/>
-      <c r="K53" s="21"/>
-      <c r="L53" s="21"/>
-      <c r="M53" s="21"/>
-      <c r="N53" s="21"/>
     </row>
     <row r="54" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G54" s="2"/>
-      <c r="H54" s="21"/>
-      <c r="I54" s="21"/>
-      <c r="J54" s="22"/>
-      <c r="K54" s="21"/>
-      <c r="L54" s="21"/>
-      <c r="M54" s="21"/>
-      <c r="N54" s="21"/>
     </row>
     <row r="55" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G55" s="2"/>
-      <c r="H55" s="21"/>
-      <c r="I55" s="21"/>
-      <c r="J55" s="22"/>
-      <c r="K55" s="21"/>
-      <c r="L55" s="21"/>
-      <c r="M55" s="21"/>
-      <c r="N55" s="21"/>
-    </row>
-    <row r="56" spans="4:14" x14ac:dyDescent="0.2">
-      <c r="H56" s="21"/>
-      <c r="I56" s="21"/>
-      <c r="J56" s="22"/>
-      <c r="K56" s="21"/>
-      <c r="L56" s="21"/>
-      <c r="M56" s="21"/>
-      <c r="N56" s="21"/>
-    </row>
-    <row r="57" spans="4:14" x14ac:dyDescent="0.2">
-      <c r="H57" s="21"/>
-      <c r="I57" s="21"/>
-      <c r="J57" s="22"/>
-      <c r="K57" s="21"/>
-      <c r="L57" s="21"/>
-      <c r="M57" s="21"/>
-      <c r="N57" s="21"/>
-    </row>
-    <row r="58" spans="4:14" x14ac:dyDescent="0.2">
-      <c r="H58" s="21"/>
-      <c r="I58" s="21"/>
-      <c r="J58" s="22"/>
-      <c r="K58" s="21"/>
-      <c r="L58" s="21"/>
-      <c r="M58" s="21"/>
-      <c r="N58" s="21"/>
     </row>
   </sheetData>
-  <autoFilter ref="D1:N47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="D1:N47" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Oui"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>

</xml_diff>

<commit_message>
erreur commit fichier temporaire
</commit_message>
<xml_diff>
--- a/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
+++ b/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Documents/Formation AI Engineer OC/Projet_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0068F7B-D0DA-AD49-A771-D782B6E289E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8262357D-19B2-1645-A008-CB8310A0C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Dictionnaire des Données" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dictionnaire des Données'!$D$1:$N$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dictionnaire des Données'!$D$1:$M$47</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="165">
   <si>
     <t>#</t>
   </si>
@@ -398,13 +398,6 @@
   </si>
   <si>
     <t xml:space="preserve">min-max scaling </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Min / Max / 
-Moy / Med </t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>FE1</t>
@@ -795,7 +788,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -846,9 +839,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -863,20 +853,17 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1180,8 +1167,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:N55"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -1192,19 +1178,18 @@
     <col min="6" max="6" width="76" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3.83203125" style="10" customWidth="1"/>
     <col min="8" max="8" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.1640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="45.1640625" customWidth="1"/>
-    <col min="13" max="13" width="29.1640625" customWidth="1"/>
-    <col min="14" max="14" width="17.1640625" customWidth="1"/>
+    <col min="9" max="9" width="32.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="45.1640625" customWidth="1"/>
+    <col min="12" max="12" width="29.1640625" customWidth="1"/>
+    <col min="13" max="13" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="35" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="24"/>
+      <c r="B1" s="25"/>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1219,30 +1204,27 @@
         <v>3</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="J1" s="13" t="s">
         <v>120</v>
       </c>
+      <c r="J1" s="9" t="s">
+        <v>134</v>
+      </c>
       <c r="K1" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="M1" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="N1" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="M1" s="9" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -1258,17 +1240,16 @@
         <v>6</v>
       </c>
       <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-    </row>
-    <row r="3" spans="1:14" ht="59" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+    </row>
+    <row r="3" spans="1:13" ht="59" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>112</v>
       </c>
@@ -1288,22 +1269,21 @@
       <c r="H3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="15"/>
-      <c r="J3" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="K3" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L3" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-    </row>
-    <row r="4" spans="1:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="I3" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+    </row>
+    <row r="4" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B4" s="8">
         <v>1668</v>
@@ -1322,19 +1302,18 @@
         <v>118</v>
       </c>
       <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L4" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-    </row>
-    <row r="5" spans="1:14" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J4" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+    </row>
+    <row r="5" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B5" s="8">
         <v>15</v>
@@ -1353,22 +1332,21 @@
         <v>12</v>
       </c>
       <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L5" s="18" t="s">
-        <v>140</v>
-      </c>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-    </row>
-    <row r="6" spans="1:14" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J5" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+    </row>
+    <row r="6" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D6" s="3">
         <v>5</v>
@@ -1384,17 +1362,16 @@
         <v>12</v>
       </c>
       <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-    </row>
-    <row r="7" spans="1:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J6" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
+    </row>
+    <row r="7" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D7" s="5">
         <v>6</v>
       </c>
@@ -1409,17 +1386,16 @@
         <v>12</v>
       </c>
       <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-    </row>
-    <row r="8" spans="1:14" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J7" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
+    </row>
+    <row r="8" spans="1:13" ht="45" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D8" s="3">
         <v>7</v>
       </c>
@@ -1434,17 +1410,16 @@
         <v>12</v>
       </c>
       <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>144</v>
-      </c>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
-    </row>
-    <row r="9" spans="1:14" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J8" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
+    </row>
+    <row r="9" spans="1:13" ht="45" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D9" s="5">
         <v>8</v>
       </c>
@@ -1459,17 +1434,16 @@
         <v>12</v>
       </c>
       <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L9" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
-    </row>
-    <row r="10" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J9" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="L9" s="17"/>
+      <c r="M9" s="17"/>
+    </row>
+    <row r="10" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D10" s="3">
         <v>9</v>
       </c>
@@ -1484,17 +1458,16 @@
         <v>12</v>
       </c>
       <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L10" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-    </row>
-    <row r="11" spans="1:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J10" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+    </row>
+    <row r="11" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D11" s="5">
         <v>10</v>
       </c>
@@ -1509,17 +1482,16 @@
         <v>12</v>
       </c>
       <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L11" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-    </row>
-    <row r="12" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J11" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+    </row>
+    <row r="12" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D12" s="3">
         <v>11</v>
       </c>
@@ -1534,17 +1506,16 @@
         <v>29</v>
       </c>
       <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L12" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-    </row>
-    <row r="13" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J12" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
+    </row>
+    <row r="13" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D13" s="5">
         <v>12</v>
       </c>
@@ -1559,17 +1530,16 @@
         <v>12</v>
       </c>
       <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L13" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-    </row>
-    <row r="14" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J13" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="L13" s="17"/>
+      <c r="M13" s="17"/>
+    </row>
+    <row r="14" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D14" s="3">
         <v>13</v>
       </c>
@@ -1584,17 +1554,16 @@
         <v>34</v>
       </c>
       <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L14" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-    </row>
-    <row r="15" spans="1:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J14" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+    </row>
+    <row r="15" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D15" s="5">
         <v>14</v>
       </c>
@@ -1609,17 +1578,16 @@
         <v>34</v>
       </c>
       <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L15" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-    </row>
-    <row r="16" spans="1:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J15" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="L15" s="17"/>
+      <c r="M15" s="17"/>
+    </row>
+    <row r="16" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="3">
         <v>15</v>
       </c>
@@ -1633,20 +1601,19 @@
       <c r="H16" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="I16" s="17"/>
-      <c r="J16" s="18" t="s">
+      <c r="I16" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="K16" s="18" t="s">
+      <c r="J16" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18" t="s">
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="5">
         <v>16</v>
       </c>
@@ -1660,20 +1627,19 @@
       <c r="H17" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="I17" s="17"/>
-      <c r="J17" s="18" t="s">
+      <c r="I17" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="J17" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18" t="s">
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D18" s="3">
         <v>17</v>
       </c>
@@ -1687,20 +1653,19 @@
       <c r="H18" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="I18" s="17"/>
-      <c r="J18" s="18" t="s">
+      <c r="I18" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K18" s="18" t="s">
+      <c r="J18" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18" t="s">
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D19" s="5">
         <v>18</v>
       </c>
@@ -1715,17 +1680,16 @@
         <v>45</v>
       </c>
       <c r="I19" s="17"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18" t="s">
+      <c r="J19" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18" t="s">
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D20" s="3">
         <v>19</v>
       </c>
@@ -1740,17 +1704,16 @@
         <v>45</v>
       </c>
       <c r="I20" s="17"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18" t="s">
+      <c r="J20" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18" t="s">
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="21" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:13" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D21" s="5">
         <v>20</v>
       </c>
@@ -1765,17 +1728,16 @@
         <v>45</v>
       </c>
       <c r="I21" s="17"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18" t="s">
+      <c r="J21" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18" t="s">
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D22" s="3">
         <v>21</v>
       </c>
@@ -1790,21 +1752,18 @@
         <v>119</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="J22" s="18" t="s">
-        <v>133</v>
-      </c>
-      <c r="K22" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="J22" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="N22" s="18"/>
-    </row>
-    <row r="23" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K22" s="17"/>
+      <c r="L22" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="M22" s="17"/>
+    </row>
+    <row r="23" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D23" s="5">
         <v>22</v>
       </c>
@@ -1819,17 +1778,16 @@
         <v>12</v>
       </c>
       <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L23" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-    </row>
-    <row r="24" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J23" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+    </row>
+    <row r="24" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D24" s="3">
         <v>23</v>
       </c>
@@ -1844,17 +1802,16 @@
         <v>45</v>
       </c>
       <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L24" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-    </row>
-    <row r="25" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J24" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K24" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+    </row>
+    <row r="25" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D25" s="5">
         <v>24</v>
       </c>
@@ -1869,17 +1826,16 @@
         <v>12</v>
       </c>
       <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L25" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M25" s="18"/>
-      <c r="N25" s="18"/>
-    </row>
-    <row r="26" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J25" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+    </row>
+    <row r="26" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D26" s="3">
         <v>25</v>
       </c>
@@ -1894,17 +1850,16 @@
         <v>45</v>
       </c>
       <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L26" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M26" s="18"/>
-      <c r="N26" s="18"/>
-    </row>
-    <row r="27" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J26" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+    </row>
+    <row r="27" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D27" s="5">
         <v>26</v>
       </c>
@@ -1919,17 +1874,16 @@
         <v>12</v>
       </c>
       <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
-      <c r="K27" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L27" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M27" s="18"/>
-      <c r="N27" s="18"/>
-    </row>
-    <row r="28" spans="4:14" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J27" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L27" s="17"/>
+      <c r="M27" s="17"/>
+    </row>
+    <row r="28" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D28" s="3">
         <v>27</v>
       </c>
@@ -1944,17 +1898,16 @@
         <v>45</v>
       </c>
       <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L28" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-    </row>
-    <row r="29" spans="4:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J28" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="L28" s="17"/>
+      <c r="M28" s="17"/>
+    </row>
+    <row r="29" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D29" s="5">
         <v>28</v>
       </c>
@@ -1969,17 +1922,16 @@
         <v>66</v>
       </c>
       <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L29" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-    </row>
-    <row r="30" spans="4:14" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J29" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+    </row>
+    <row r="30" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D30" s="3">
         <v>29</v>
       </c>
@@ -1994,17 +1946,16 @@
         <v>69</v>
       </c>
       <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-      <c r="K30" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L30" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="M30" s="18"/>
-      <c r="N30" s="18"/>
-    </row>
-    <row r="31" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J30" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="L30" s="17"/>
+      <c r="M30" s="17"/>
+    </row>
+    <row r="31" spans="4:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D31" s="5">
         <v>30</v>
       </c>
@@ -2019,17 +1970,16 @@
         <v>72</v>
       </c>
       <c r="I31" s="17"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18" t="s">
+      <c r="J31" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
-      <c r="N31" s="18" t="s">
+      <c r="K31" s="17"/>
+      <c r="L31" s="17"/>
+      <c r="M31" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D32" s="3">
         <v>31</v>
       </c>
@@ -2044,17 +1994,16 @@
         <v>72</v>
       </c>
       <c r="I32" s="15"/>
-      <c r="J32" s="15"/>
-      <c r="K32" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L32" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-    </row>
-    <row r="33" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J32" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
+    </row>
+    <row r="33" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D33" s="5">
         <v>32</v>
       </c>
@@ -2069,17 +2018,16 @@
         <v>72</v>
       </c>
       <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
-      <c r="K33" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L33" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="M33" s="18"/>
-      <c r="N33" s="18"/>
-    </row>
-    <row r="34" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J33" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+    </row>
+    <row r="34" spans="4:13" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D34" s="3">
         <v>33</v>
       </c>
@@ -2094,17 +2042,16 @@
         <v>72</v>
       </c>
       <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L34" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="M34" s="18"/>
-      <c r="N34" s="18"/>
-    </row>
-    <row r="35" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J34" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K34" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="L34" s="17"/>
+      <c r="M34" s="17"/>
+    </row>
+    <row r="35" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D35" s="5">
         <v>34</v>
       </c>
@@ -2118,22 +2065,21 @@
       <c r="H35" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I35" s="17"/>
-      <c r="J35" s="18" t="s">
+      <c r="I35" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K35" s="18" t="s">
+      <c r="J35" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18" t="s">
+      <c r="K35" s="17"/>
+      <c r="L35" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N35" s="27" t="s">
+      <c r="M35" s="23" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D36" s="3">
         <v>35</v>
       </c>
@@ -2148,17 +2094,16 @@
         <v>81</v>
       </c>
       <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
-      <c r="K36" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L36" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="M36" s="18"/>
-      <c r="N36" s="18"/>
-    </row>
-    <row r="37" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J36" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+    </row>
+    <row r="37" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D37" s="5">
         <v>36</v>
       </c>
@@ -2172,20 +2117,19 @@
       <c r="H37" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I37" s="17"/>
-      <c r="J37" s="18" t="s">
+      <c r="I37" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K37" s="18" t="s">
+      <c r="J37" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L37" s="18"/>
-      <c r="M37" s="18"/>
-      <c r="N37" s="18" t="s">
+      <c r="K37" s="17"/>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D38" s="3">
         <v>37</v>
       </c>
@@ -2200,17 +2144,16 @@
         <v>88</v>
       </c>
       <c r="I38" s="15"/>
-      <c r="J38" s="15"/>
-      <c r="K38" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L38" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="M38" s="18"/>
-      <c r="N38" s="18"/>
-    </row>
-    <row r="39" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J38" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K38" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+    </row>
+    <row r="39" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D39" s="5">
         <v>38</v>
       </c>
@@ -2224,20 +2167,19 @@
       <c r="H39" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I39" s="17"/>
-      <c r="J39" s="18" t="s">
+      <c r="I39" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K39" s="18" t="s">
+      <c r="J39" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L39" s="18"/>
-      <c r="M39" s="18"/>
-      <c r="N39" s="18" t="s">
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D40" s="3">
         <v>39</v>
       </c>
@@ -2252,17 +2194,16 @@
         <v>93</v>
       </c>
       <c r="I40" s="15"/>
-      <c r="J40" s="15"/>
-      <c r="K40" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L40" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="M40" s="18"/>
-      <c r="N40" s="18"/>
-    </row>
-    <row r="41" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J40" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K40" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="L40" s="17"/>
+      <c r="M40" s="17"/>
+    </row>
+    <row r="41" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D41" s="5">
         <v>40</v>
       </c>
@@ -2276,20 +2217,19 @@
       <c r="H41" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I41" s="17"/>
-      <c r="J41" s="18" t="s">
+      <c r="I41" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="K41" s="18" t="s">
+      <c r="J41" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L41" s="18"/>
-      <c r="M41" s="18"/>
-      <c r="N41" s="18" t="s">
+      <c r="K41" s="17"/>
+      <c r="L41" s="17"/>
+      <c r="M41" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D42" s="3">
         <v>41</v>
       </c>
@@ -2303,20 +2243,19 @@
       <c r="H42" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="I42" s="17"/>
-      <c r="J42" s="18" t="s">
+      <c r="I42" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="K42" s="18" t="s">
+      <c r="J42" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L42" s="18"/>
-      <c r="M42" s="18"/>
-      <c r="N42" s="18" t="s">
+      <c r="K42" s="17"/>
+      <c r="L42" s="17"/>
+      <c r="M42" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="43" spans="4:14" ht="28" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:13" ht="28" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D43" s="5">
         <v>42</v>
       </c>
@@ -2331,17 +2270,16 @@
         <v>12</v>
       </c>
       <c r="I43" s="15"/>
-      <c r="J43" s="15"/>
-      <c r="K43" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L43" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="M43" s="18"/>
-      <c r="N43" s="18"/>
-    </row>
-    <row r="44" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J43" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K43" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="L43" s="17"/>
+      <c r="M43" s="17"/>
+    </row>
+    <row r="44" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D44" s="3">
         <v>43</v>
       </c>
@@ -2356,21 +2294,18 @@
         <v>119</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="J44" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="K44" s="18" t="s">
+      <c r="J44" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L44" s="18"/>
-      <c r="M44" s="18"/>
-      <c r="N44" s="18" t="s">
+      <c r="K44" s="17"/>
+      <c r="L44" s="17"/>
+      <c r="M44" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D45" s="5">
         <v>44</v>
       </c>
@@ -2384,22 +2319,21 @@
       <c r="H45" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="I45" s="17"/>
-      <c r="J45" s="18" t="s">
+      <c r="I45" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="K45" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L45" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="M45" s="18"/>
-      <c r="N45" s="18" t="s">
+      <c r="J45" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K45" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="L45" s="17"/>
+      <c r="M45" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="46" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D46" s="3">
         <v>45</v>
       </c>
@@ -2414,19 +2348,18 @@
         <v>107</v>
       </c>
       <c r="I46" s="17"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18" t="s">
+      <c r="J46" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L46" s="18"/>
-      <c r="M46" s="18" t="s">
+      <c r="K46" s="17"/>
+      <c r="L46" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N46" s="18" t="s">
+      <c r="M46" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="4:14" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D47" s="5">
         <v>46</v>
       </c>
@@ -2441,17 +2374,16 @@
         <v>110</v>
       </c>
       <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L47" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="M47" s="18"/>
-      <c r="N47" s="18"/>
-    </row>
-    <row r="48" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J47" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K47" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="L47" s="17"/>
+      <c r="M47" s="17"/>
+    </row>
+    <row r="48" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
@@ -2462,89 +2394,82 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
-      <c r="N48" s="2"/>
-    </row>
-    <row r="49" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D49" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="E49" s="20" t="s">
-        <v>166</v>
-      </c>
-      <c r="F49" s="21" t="s">
-        <v>130</v>
+    </row>
+    <row r="49" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D49" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="F49" s="20" t="s">
+        <v>128</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="J49" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="K49" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="I49" s="17" t="s">
+        <v>129</v>
+      </c>
+      <c r="J49" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L49" s="18"/>
-      <c r="M49" s="18" t="s">
+      <c r="K49" s="17"/>
+      <c r="L49" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N49" s="18" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="50" spans="4:14" ht="31" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D50" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="E50" s="20" t="s">
-        <v>135</v>
-      </c>
-      <c r="F50" s="21" t="s">
-        <v>156</v>
+      <c r="M49" s="17" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="50" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D50" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="F50" s="20" t="s">
+        <v>154</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="J50" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="K50" s="18" t="s">
+      <c r="I50" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="J50" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="L50" s="18"/>
-      <c r="M50" s="18" t="s">
+      <c r="K50" s="17"/>
+      <c r="L50" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="N50" s="18" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="51" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M50" s="17" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G51" s="2"/>
-      <c r="H51" s="25"/>
-      <c r="K51" s="26"/>
-    </row>
-    <row r="52" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H51" s="22"/>
+      <c r="J51" s="17"/>
+    </row>
+    <row r="52" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G52" s="2"/>
     </row>
-    <row r="53" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G53" s="2"/>
     </row>
-    <row r="54" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G54" s="2"/>
     </row>
-    <row r="55" spans="4:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G55" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="D1:N47" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="7">
-      <filters>
-        <filter val="Oui"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="D1:M47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Début du Feature Engineering
</commit_message>
<xml_diff>
--- a/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
+++ b/OC_P3_ Seattle_Building_Energy_Benchmarking_Columns-v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Documents/Formation AI Engineer OC/Projet_3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8262357D-19B2-1645-A008-CB8310A0C329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CDEF20-2B57-5C41-99F8-FC450AC58C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Dictionnaire des Données" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dictionnaire des Données'!$D$1:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dictionnaire des Données'!$D$1:$L$47</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="166">
   <si>
     <t>#</t>
   </si>
@@ -394,9 +394,6 @@
     <t>Convertir en binaire numérique pour le modele</t>
   </si>
   <si>
-    <t>One hot encoding</t>
-  </si>
-  <si>
     <t xml:space="preserve">min-max scaling </t>
   </si>
   <si>
@@ -413,9 +410,6 @@
   </si>
   <si>
     <t>Calculée a partir du nb de valeurs dans la variable "ListOfAllPropertyUseTypes"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Garder pour entrainnement du modele </t>
   </si>
   <si>
     <t>Pour alimenter FE1</t>
@@ -602,6 +596,15 @@
   </si>
   <si>
     <t xml:space="preserve">Is_multi_type </t>
+  </si>
+  <si>
+    <t>FE3</t>
+  </si>
+  <si>
+    <t>FE4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pas pertinent pour l'analyse ou le ML </t>
   </si>
 </sst>
 </file>
@@ -788,7 +791,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -849,9 +852,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1167,7 +1167,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M55"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -1181,15 +1182,14 @@
     <col min="9" max="9" width="32.1640625" style="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20.83203125" customWidth="1"/>
     <col min="11" max="11" width="45.1640625" customWidth="1"/>
-    <col min="12" max="12" width="29.1640625" customWidth="1"/>
-    <col min="13" max="13" width="17.1640625" customWidth="1"/>
+    <col min="12" max="12" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:12" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="25"/>
+      <c r="B1" s="24"/>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1207,24 +1207,21 @@
         <v>120</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="M1" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="L1" s="9" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
@@ -1244,12 +1241,11 @@
         <v>114</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-    </row>
-    <row r="3" spans="1:13" ht="59" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:12" ht="59" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>112</v>
       </c>
@@ -1270,20 +1266,19 @@
         <v>9</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J3" s="17" t="s">
         <v>114</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-    </row>
-    <row r="4" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B4" s="8">
         <v>1668</v>
@@ -1306,14 +1301,13 @@
         <v>114</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-    </row>
-    <row r="5" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:12" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B5" s="8">
         <v>15</v>
@@ -1336,17 +1330,16 @@
         <v>114</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-    </row>
-    <row r="6" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:12" ht="33" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D6" s="3">
         <v>5</v>
@@ -1366,12 +1359,11 @@
         <v>114</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-    </row>
-    <row r="7" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:12" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D7" s="5">
         <v>6</v>
       </c>
@@ -1390,12 +1382,11 @@
         <v>114</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-    </row>
-    <row r="8" spans="1:13" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:12" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D8" s="3">
         <v>7</v>
       </c>
@@ -1414,12 +1405,11 @@
         <v>114</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-    </row>
-    <row r="9" spans="1:13" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:12" ht="45" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D9" s="5">
         <v>8</v>
       </c>
@@ -1438,12 +1428,11 @@
         <v>114</v>
       </c>
       <c r="K9" s="17" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-    </row>
-    <row r="10" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D10" s="3">
         <v>9</v>
       </c>
@@ -1462,12 +1451,11 @@
         <v>114</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-    </row>
-    <row r="11" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:12" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D11" s="5">
         <v>10</v>
       </c>
@@ -1486,12 +1474,11 @@
         <v>114</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-    </row>
-    <row r="12" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D12" s="3">
         <v>11</v>
       </c>
@@ -1510,12 +1497,11 @@
         <v>114</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-    </row>
-    <row r="13" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D13" s="5">
         <v>12</v>
       </c>
@@ -1527,19 +1513,20 @@
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="15"/>
+        <v>119</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>122</v>
+      </c>
       <c r="J13" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
-    </row>
-    <row r="14" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D14" s="3">
         <v>13</v>
       </c>
@@ -1558,12 +1545,11 @@
         <v>114</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-    </row>
-    <row r="15" spans="1:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D15" s="5">
         <v>14</v>
       </c>
@@ -1582,12 +1568,11 @@
         <v>114</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-    </row>
-    <row r="16" spans="1:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:12" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="3">
         <v>15</v>
       </c>
@@ -1608,12 +1593,11 @@
         <v>115</v>
       </c>
       <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17" t="s">
+      <c r="L16" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="5">
         <v>16</v>
       </c>
@@ -1628,18 +1612,17 @@
         <v>29</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J17" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17" t="s">
+      <c r="L17" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="18" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D18" s="3">
         <v>17</v>
       </c>
@@ -1654,18 +1637,17 @@
         <v>29</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J18" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17" t="s">
+      <c r="L18" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:12" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D19" s="5">
         <v>18</v>
       </c>
@@ -1684,12 +1666,11 @@
         <v>115</v>
       </c>
       <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17" t="s">
+      <c r="L19" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="20" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D20" s="3">
         <v>19</v>
       </c>
@@ -1708,12 +1689,11 @@
         <v>115</v>
       </c>
       <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17" t="s">
+      <c r="L20" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="21" spans="4:13" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:12" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D21" s="5">
         <v>20</v>
       </c>
@@ -1732,12 +1712,11 @@
         <v>115</v>
       </c>
       <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17" t="s">
+      <c r="L21" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D22" s="3">
         <v>21</v>
       </c>
@@ -1752,18 +1731,15 @@
         <v>119</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K22" s="17"/>
-      <c r="L22" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="M22" s="17"/>
-    </row>
-    <row r="23" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L22" s="17"/>
+    </row>
+    <row r="23" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D23" s="5">
         <v>22</v>
       </c>
@@ -1782,12 +1758,11 @@
         <v>114</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-    </row>
-    <row r="24" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D24" s="3">
         <v>23</v>
       </c>
@@ -1806,12 +1781,11 @@
         <v>114</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L24" s="17"/>
-      <c r="M24" s="17"/>
-    </row>
-    <row r="25" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D25" s="5">
         <v>24</v>
       </c>
@@ -1830,12 +1804,11 @@
         <v>114</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-    </row>
-    <row r="26" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D26" s="3">
         <v>25</v>
       </c>
@@ -1854,12 +1827,11 @@
         <v>114</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
-    </row>
-    <row r="27" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D27" s="5">
         <v>26</v>
       </c>
@@ -1878,12 +1850,11 @@
         <v>114</v>
       </c>
       <c r="K27" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L27" s="17"/>
-      <c r="M27" s="17"/>
-    </row>
-    <row r="28" spans="4:13" ht="46" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="4:12" ht="46" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D28" s="3">
         <v>27</v>
       </c>
@@ -1902,12 +1873,11 @@
         <v>114</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
-    </row>
-    <row r="29" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="4:12" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D29" s="5">
         <v>28</v>
       </c>
@@ -1926,12 +1896,11 @@
         <v>114</v>
       </c>
       <c r="K29" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-    </row>
-    <row r="30" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="4:12" ht="17" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D30" s="3">
         <v>29</v>
       </c>
@@ -1950,12 +1919,11 @@
         <v>114</v>
       </c>
       <c r="K30" s="17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L30" s="17"/>
-      <c r="M30" s="17"/>
-    </row>
-    <row r="31" spans="4:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="4:12" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D31" s="5">
         <v>30</v>
       </c>
@@ -1974,12 +1942,11 @@
         <v>115</v>
       </c>
       <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
-      <c r="M31" s="17" t="s">
+      <c r="L31" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D32" s="3">
         <v>31</v>
       </c>
@@ -1998,12 +1965,11 @@
         <v>114</v>
       </c>
       <c r="K32" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L32" s="17"/>
-      <c r="M32" s="17"/>
-    </row>
-    <row r="33" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D33" s="5">
         <v>32</v>
       </c>
@@ -2022,12 +1988,11 @@
         <v>114</v>
       </c>
       <c r="K33" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-    </row>
-    <row r="34" spans="4:13" ht="38" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="4:12" ht="38" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D34" s="3">
         <v>33</v>
       </c>
@@ -2046,12 +2011,11 @@
         <v>114</v>
       </c>
       <c r="K34" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L34" s="17"/>
-      <c r="M34" s="17"/>
-    </row>
-    <row r="35" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D35" s="5">
         <v>34</v>
       </c>
@@ -2066,20 +2030,17 @@
         <v>81</v>
       </c>
       <c r="I35" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J35" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K35" s="17"/>
-      <c r="L35" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="M35" s="23" t="s">
+      <c r="L35" s="22" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D36" s="3">
         <v>35</v>
       </c>
@@ -2098,12 +2059,11 @@
         <v>114</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-    </row>
-    <row r="37" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D37" s="5">
         <v>36</v>
       </c>
@@ -2118,18 +2078,17 @@
         <v>81</v>
       </c>
       <c r="I37" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J37" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17" t="s">
+      <c r="L37" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="38" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D38" s="3">
         <v>37</v>
       </c>
@@ -2148,12 +2107,11 @@
         <v>114</v>
       </c>
       <c r="K38" s="17" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-    </row>
-    <row r="39" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D39" s="5">
         <v>38</v>
       </c>
@@ -2168,18 +2126,17 @@
         <v>81</v>
       </c>
       <c r="I39" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J39" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
-      <c r="M39" s="17" t="s">
+      <c r="L39" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D40" s="3">
         <v>39</v>
       </c>
@@ -2198,12 +2155,11 @@
         <v>114</v>
       </c>
       <c r="K40" s="17" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L40" s="17"/>
-      <c r="M40" s="17"/>
-    </row>
-    <row r="41" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D41" s="5">
         <v>40</v>
       </c>
@@ -2218,18 +2174,17 @@
         <v>81</v>
       </c>
       <c r="I41" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J41" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17" t="s">
+      <c r="L41" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="42" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D42" s="3">
         <v>41</v>
       </c>
@@ -2243,19 +2198,18 @@
       <c r="H42" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="I42" s="17" t="s">
-        <v>122</v>
-      </c>
+      <c r="I42" s="17"/>
       <c r="J42" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="K42" s="17"/>
-      <c r="L42" s="17"/>
-      <c r="M42" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K42" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="L42" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="43" spans="4:13" ht="28" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:12" ht="28" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D43" s="5">
         <v>42</v>
       </c>
@@ -2274,12 +2228,11 @@
         <v>114</v>
       </c>
       <c r="K43" s="17" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-    </row>
-    <row r="44" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D44" s="3">
         <v>43</v>
       </c>
@@ -2293,19 +2246,18 @@
       <c r="H44" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="I44" s="17" t="s">
-        <v>123</v>
-      </c>
+      <c r="I44" s="17"/>
       <c r="J44" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="K44" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="L44" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D45" s="5">
         <v>44</v>
       </c>
@@ -2326,14 +2278,13 @@
         <v>114</v>
       </c>
       <c r="K45" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="L45" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="46" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:12" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D46" s="3">
         <v>45</v>
       </c>
@@ -2353,13 +2304,10 @@
       </c>
       <c r="K46" s="17"/>
       <c r="L46" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="M46" s="17" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="47" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:12" ht="31" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D47" s="5">
         <v>46</v>
       </c>
@@ -2378,12 +2326,11 @@
         <v>114</v>
       </c>
       <c r="K47" s="17" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-    </row>
-    <row r="48" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
@@ -2393,83 +2340,103 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
-    </row>
-    <row r="49" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="4:12" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D49" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E49" s="19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F49" s="20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I49" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J49" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K49" s="17"/>
       <c r="L49" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="M49" s="17" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="50" spans="4:13" ht="31" thickBot="1" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="4:12" ht="31" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D50" s="18" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F50" s="20" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="16" t="s">
         <v>9</v>
       </c>
       <c r="I50" s="17" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="J50" s="17" t="s">
         <v>115</v>
       </c>
       <c r="K50" s="17"/>
       <c r="L50" s="17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="51" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D51" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E51" s="19"/>
+      <c r="F51" s="20"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="21"/>
+      <c r="J51" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="M50" s="17" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="51" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G51" s="2"/>
-      <c r="H51" s="22"/>
-      <c r="J51" s="17"/>
-    </row>
-    <row r="52" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L51" s="17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="52" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D52" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="E52" s="19"/>
+      <c r="F52" s="20"/>
       <c r="G52" s="2"/>
-    </row>
-    <row r="53" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J52" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="L52" s="17" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="53" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G53" s="2"/>
     </row>
-    <row r="54" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G54" s="2"/>
     </row>
-    <row r="55" spans="4:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G55" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="D1:M47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="D1:L47" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Oui"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>

</xml_diff>